<commit_message>
corrected some template formatting
</commit_message>
<xml_diff>
--- a/templates/HEM4_Emiss_Loc_ICF.xlsx
+++ b/templates/HEM4_Emiss_Loc_ICF.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\HEM4 Home\HEM4 Inputs\Intl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55586\Desktop\tools\access tool\access-tool-migration\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4381DD-5846-4023-BB05-11983DB2838A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3B88B8-48D1-4EA6-978C-8683C764E3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1980" yWindow="600" windowWidth="21060" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7305" yWindow="2700" windowWidth="26265" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Emissions_Location" sheetId="1" r:id="rId1"/>
@@ -316,7 +316,7 @@
     <numFmt numFmtId="164" formatCode="0.0000000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Arial"/>
@@ -328,11 +328,6 @@
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -373,20 +368,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -401,18 +395,18 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -539,9 +533,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -579,9 +573,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -614,26 +608,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -666,26 +643,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -927,132 +887,132 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:IV4"/>
-  <sheetFormatPr defaultColWidth="7.6796875" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="7.6640625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.86328125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="8.6796875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.76953125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="18.31640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="20.08984375" style="4" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.2265625" style="3" customWidth="1"/>
-    <col min="8" max="9" width="9.6796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" style="4" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" style="3" customWidth="1"/>
+    <col min="8" max="9" width="9.6640625" style="3" customWidth="1"/>
     <col min="10" max="10" width="10" style="3" customWidth="1"/>
-    <col min="11" max="11" width="10.31640625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="10.6796875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="15.31640625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="9.6796875" style="5" customWidth="1"/>
-    <col min="15" max="15" width="8.54296875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="8.31640625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="9.86328125" style="2" customWidth="1"/>
-    <col min="18" max="18" width="7.6796875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="15.76953125" style="2" customWidth="1"/>
-    <col min="20" max="20" width="13.86328125" style="2" customWidth="1"/>
-    <col min="21" max="16384" width="7.6796875" style="2"/>
+    <col min="11" max="11" width="10.33203125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="10.6640625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="15.33203125" style="3" customWidth="1"/>
+    <col min="14" max="14" width="9.6640625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="8.5546875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="8.33203125" style="2" customWidth="1"/>
+    <col min="17" max="17" width="9.88671875" style="2" customWidth="1"/>
+    <col min="18" max="18" width="7.6640625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="15.77734375" style="2" customWidth="1"/>
+    <col min="20" max="20" width="13.88671875" style="2" customWidth="1"/>
+    <col min="21" max="16384" width="7.6640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:256" s="13" customFormat="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="15"/>
-      <c r="C1" s="16" t="s">
+    <row r="1" spans="1:256" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="14"/>
+      <c r="C1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="16" t="s">
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="17" t="s">
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="15"/>
-      <c r="S1" s="18" t="s">
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="18"/>
-      <c r="U1" s="16" t="s">
+      <c r="T1" s="17"/>
+      <c r="U1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
+      <c r="V1" s="15"/>
+      <c r="W1" s="15"/>
     </row>
-    <row r="2" spans="1:256" ht="36.9" x14ac:dyDescent="0.4">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:256" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="K2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="L2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="R2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="S2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="T2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="U2" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="8" t="s">
+      <c r="V2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="W2" s="8" t="s">
+      <c r="W2" s="7" t="s">
         <v>26</v>
       </c>
       <c r="X2" s="1"/>
@@ -1289,9 +1249,9 @@
       <c r="IU2" s="1"/>
       <c r="IV2" s="1"/>
     </row>
-    <row r="4" spans="1:256" x14ac:dyDescent="0.4">
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
+    <row r="4" spans="1:256" x14ac:dyDescent="0.2">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1312,7 +1272,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BFB2418-13A9-4239-A583-B90637E81481}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1329,6 +1289,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010071E84B6C57E3394DA6F02D58EDB00D49" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bcbb874a66251b8305a28e53f7e58f29">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bf1cdca2-fdad-4885-8dd1-8619069b9665" xmlns:ns3="29780eff-3761-499e-ba1f-97668a174bb3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9e6e6b42b6445f8c6c2f2438f079088d" ns2:_="" ns3:_="">
     <xsd:import namespace="bf1cdca2-fdad-4885-8dd1-8619069b9665"/>
@@ -1493,12 +1459,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F32BA10E-D1BC-49EE-9CB1-FC8D8B309A82}">
   <ds:schemaRefs>
@@ -1508,6 +1468,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B592FEAF-C5E9-4AB9-9C35-46CA833370EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2ABC03AD-88D9-4E2C-AC0F-EDE0445632D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1524,13 +1493,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B592FEAF-C5E9-4AB9-9C35-46CA833370EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
corrected file naming and accdb access
</commit_message>
<xml_diff>
--- a/templates/HEM4_Emiss_Loc_ICF.xlsx
+++ b/templates/HEM4_Emiss_Loc_ICF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55586\Desktop\tools\access tool\access-tool-migration\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3B88B8-48D1-4EA6-978C-8683C764E3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B5C969B-A78F-436E-AA4C-A17A74977D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7305" yWindow="2700" windowWidth="26265" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6465" yWindow="2130" windowWidth="26265" windowHeight="15060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Emissions_Location" sheetId="1" r:id="rId1"/>
@@ -368,19 +368,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -395,20 +395,21 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -912,14 +913,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:256" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14"/>
+      <c r="A1" s="13"/>
       <c r="C1" s="15" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
       <c r="F1" s="15"/>
-      <c r="G1" s="13"/>
+      <c r="G1" s="14"/>
       <c r="H1" s="15" t="s">
         <v>3</v>
       </c>
@@ -934,7 +935,7 @@
       <c r="O1" s="16"/>
       <c r="P1" s="16"/>
       <c r="Q1" s="16"/>
-      <c r="R1" s="14"/>
+      <c r="R1" s="13"/>
       <c r="S1" s="17" t="s">
         <v>5</v>
       </c>
@@ -1250,8 +1251,8 @@
       <c r="IV2" s="1"/>
     </row>
     <row r="4" spans="1:256" x14ac:dyDescent="0.2">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>